<commit_message>
Agrega pruebas y completa la documentacion del proyecto
</commit_message>
<xml_diff>
--- a/data/raw/datos 2022 y 2026.xlsx
+++ b/data/raw/datos 2022 y 2026.xlsx
@@ -152,7 +152,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartidosMundiales2022y2026" displayName="PartidosMundiales2022y2026" ref="A1:O168" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartidosMundiales2022y2026" displayName="PartidosMundiales2022y2026" ref="A1:O169" headerRowCount="1">
   <autoFilter ref="A1:O168"/>
   <tableColumns count="15">
     <tableColumn id="1" name="year"/>
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6">
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7">
@@ -537,8 +537,8 @@
           <t>?ltima fecha incluida</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
-        <v>46221.5</v>
+      <c r="B8" s="4" t="n">
+        <v>46222</v>
       </c>
     </row>
     <row r="9">
@@ -547,8 +547,8 @@
           <t>Fecha de preparaci?n</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
-        <v>46222</v>
+      <c r="B9" s="4" t="n">
+        <v>46227</v>
       </c>
     </row>
     <row r="10">
@@ -559,7 +559,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Se incluyen 103 partidos finalizados hasta el 18-07-2026. La final del 19-07-2026 queda excluida por no tener resultado final al preparar el archivo.</t>
+          <t>Se incluyen los 104 partidos finalizados del Mundial 2026, incluida la final Espa?a 1-0 Argentina despu?s de tiempo extra.</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Se combinaron las hojas de partidos, se conservaron las 15 columnas y se ordenaron los registros cronol?gicamente.</t>
+          <t>Se combinaron las hojas de partidos, se conservaron las 15 columnas, se ordenaron cronol?gicamente y se agreg? la final verificada con FIFA.</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O168"/>
+  <dimension ref="A1:O169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11151,6 +11151,75 @@
         </is>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>New York/New Jersey (East Rutherford)</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="G169" t="n">
+        <v>1</v>
+      </c>
+      <c r="H169" t="n">
+        <v>0</v>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Spain won after extra time</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="M169" s="4" t="n">
+        <v>46222.5</v>
+      </c>
+      <c r="N169" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O168"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11166,7 +11235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11259,7 +11328,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>103 partidos finalizados, 11-06-2026 a 18-07-2026</t>
+          <t>104 partidos finalizados, 11-06-2026 a 19-07-2026; final incluida</t>
         </is>
       </c>
     </row>
@@ -11281,7 +11350,29 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>103 partidos finalizados; final no incluida</t>
+          <t>104 partidos finalizados, 11-06-2026 a 19-07-2026; final incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Informe oficial de la final</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/articles/spain-argentina-final-report-highlights</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Espa?a 1-0 Argentina despu?s de tiempo extra, 19-07-2026</t>
         </is>
       </c>
     </row>

</xml_diff>